<commit_message>
Added V1.0 pinmap data and update schematics
</commit_message>
<xml_diff>
--- a/Design/HLD_Design/Project_OAK_MCU_Pinouts.xlsx
+++ b/Design/HLD_Design/Project_OAK_MCU_Pinouts.xlsx
@@ -7,15 +7,16 @@
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
-    <sheet name="Pin_Mapping" sheetId="1" r:id="rId1"/>
-    <sheet name="LED_Mapping" sheetId="2" r:id="rId2"/>
+    <sheet name="Pin_Mapping_V1.0" sheetId="3" r:id="rId1"/>
+    <sheet name="Pin_Mapping_V0.1" sheetId="1" r:id="rId2"/>
+    <sheet name="LED_Mapping_V0.1" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="149">
   <si>
     <t>S. No</t>
   </si>
@@ -453,6 +454,15 @@
   </si>
   <si>
     <t>PE3</t>
+  </si>
+  <si>
+    <t>BTN + ACC_INT1</t>
+  </si>
+  <si>
+    <t>ACC_INT2</t>
+  </si>
+  <si>
+    <t>RTC + ACC</t>
   </si>
 </sst>
 </file>
@@ -483,7 +493,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -577,6 +587,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -744,7 +760,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -800,6 +816,48 @@
     <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -812,9 +870,6 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -869,33 +924,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -903,6 +931,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1199,6 +1230,839 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A2:M36"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:13">
+      <c r="A2" s="4"/>
+      <c r="B2" s="37" t="s">
+        <v>106</v>
+      </c>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
+      <c r="G2" s="37"/>
+      <c r="H2" s="37"/>
+      <c r="I2" s="37"/>
+      <c r="J2" s="37"/>
+      <c r="L2" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="M2" s="2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="4"/>
+      <c r="B3" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="32" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="29" t="s">
+        <v>92</v>
+      </c>
+      <c r="J3" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="M3" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="4"/>
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="H4" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="I4" s="29"/>
+      <c r="J4" s="29"/>
+      <c r="L4" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="M4" s="2">
+        <f>M2-M3</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="4"/>
+      <c r="B5" s="21">
+        <v>1</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="31" t="s">
+        <v>90</v>
+      </c>
+      <c r="E5" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="H5" s="21"/>
+      <c r="I5" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="4"/>
+      <c r="B6" s="21">
+        <v>2</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="30"/>
+      <c r="E6" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="19" t="s">
+        <v>100</v>
+      </c>
+      <c r="J6" s="9" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="4"/>
+      <c r="B7" s="21">
+        <v>3</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="30"/>
+      <c r="E7" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="H7" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="I7" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="J7" s="12" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="4"/>
+      <c r="B8" s="21">
+        <v>4</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="38" t="s">
+        <v>89</v>
+      </c>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="39"/>
+      <c r="I8" s="39"/>
+      <c r="J8" s="40"/>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="4"/>
+      <c r="B9" s="21">
+        <v>5</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="41"/>
+      <c r="E9" s="42"/>
+      <c r="F9" s="42"/>
+      <c r="G9" s="42"/>
+      <c r="H9" s="42"/>
+      <c r="I9" s="42"/>
+      <c r="J9" s="43"/>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10" s="4"/>
+      <c r="B10" s="21">
+        <v>6</v>
+      </c>
+      <c r="C10" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="E10" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="F10" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="G10" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="H10" s="21"/>
+      <c r="I10" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="J10" s="58" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
+      <c r="A11" s="4"/>
+      <c r="B11" s="21">
+        <v>7</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="31" t="s">
+        <v>91</v>
+      </c>
+      <c r="E11" s="30"/>
+      <c r="F11" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" s="21"/>
+      <c r="H11" s="21"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="31" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13">
+      <c r="A12" s="4"/>
+      <c r="B12" s="21">
+        <v>8</v>
+      </c>
+      <c r="C12" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" s="30"/>
+      <c r="E12" s="30"/>
+      <c r="F12" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="G12" s="21"/>
+      <c r="H12" s="21"/>
+      <c r="I12" s="28"/>
+      <c r="J12" s="31"/>
+    </row>
+    <row r="13" spans="1:13">
+      <c r="A13" s="4"/>
+      <c r="B13" s="21">
+        <v>9</v>
+      </c>
+      <c r="C13" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="31" t="s">
+        <v>90</v>
+      </c>
+      <c r="E13" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="F13" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="G13" s="21"/>
+      <c r="H13" s="21"/>
+      <c r="I13" s="19" t="s">
+        <v>100</v>
+      </c>
+      <c r="J13" s="9" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13">
+      <c r="A14" s="4"/>
+      <c r="B14" s="21">
+        <v>10</v>
+      </c>
+      <c r="C14" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="30"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="G14" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="H14" s="21"/>
+      <c r="I14" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="J14" s="33" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13">
+      <c r="A15" s="4"/>
+      <c r="B15" s="21">
+        <v>11</v>
+      </c>
+      <c r="C15" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="D15" s="30"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="G15" s="21"/>
+      <c r="H15" s="21"/>
+      <c r="I15" s="28"/>
+      <c r="J15" s="34"/>
+    </row>
+    <row r="16" spans="1:13">
+      <c r="A16" s="4"/>
+      <c r="B16" s="21">
+        <v>12</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16" s="30"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="G16" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H16" s="21"/>
+      <c r="I16" s="28"/>
+      <c r="J16" s="34"/>
+    </row>
+    <row r="17" spans="1:10">
+      <c r="A17" s="4"/>
+      <c r="B17" s="21">
+        <v>13</v>
+      </c>
+      <c r="C17" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="D17" s="30"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="G17" s="21"/>
+      <c r="H17" s="21"/>
+      <c r="I17" s="28"/>
+      <c r="J17" s="34"/>
+    </row>
+    <row r="18" spans="1:10">
+      <c r="A18" s="4"/>
+      <c r="B18" s="21">
+        <v>14</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D18" s="30"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="G18" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="H18" s="21"/>
+      <c r="I18" s="28"/>
+      <c r="J18" s="35"/>
+    </row>
+    <row r="19" spans="1:10">
+      <c r="A19" s="4"/>
+      <c r="B19" s="21">
+        <v>15</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="G19" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="H19" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="I19" s="28" t="s">
+        <v>99</v>
+      </c>
+      <c r="J19" s="51" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10">
+      <c r="A20" s="4"/>
+      <c r="B20" s="21">
+        <v>16</v>
+      </c>
+      <c r="C20" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" s="30"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="G20" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="H20" s="21"/>
+      <c r="I20" s="28"/>
+      <c r="J20" s="51"/>
+    </row>
+    <row r="21" spans="1:10">
+      <c r="A21" s="4"/>
+      <c r="B21" s="21">
+        <v>17</v>
+      </c>
+      <c r="C21" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="D21" s="30"/>
+      <c r="E21" s="30"/>
+      <c r="F21" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="G21" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="H21" s="21"/>
+      <c r="I21" s="28"/>
+      <c r="J21" s="51"/>
+    </row>
+    <row r="22" spans="1:10">
+      <c r="A22" s="4"/>
+      <c r="B22" s="21">
+        <v>18</v>
+      </c>
+      <c r="C22" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="D22" s="44" t="s">
+        <v>89</v>
+      </c>
+      <c r="E22" s="45"/>
+      <c r="F22" s="45"/>
+      <c r="G22" s="45"/>
+      <c r="H22" s="45"/>
+      <c r="I22" s="45"/>
+      <c r="J22" s="46"/>
+    </row>
+    <row r="23" spans="1:10">
+      <c r="A23" s="4"/>
+      <c r="B23" s="21">
+        <v>19</v>
+      </c>
+      <c r="C23" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="D23" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="F23" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="G23" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="H23" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="I23" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="J23" s="19" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10">
+      <c r="A24" s="4"/>
+      <c r="B24" s="21">
+        <v>20</v>
+      </c>
+      <c r="C24" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="D24" s="25" t="s">
+        <v>112</v>
+      </c>
+      <c r="E24" s="26"/>
+      <c r="F24" s="26"/>
+      <c r="G24" s="26"/>
+      <c r="H24" s="26"/>
+      <c r="I24" s="26"/>
+      <c r="J24" s="27"/>
+    </row>
+    <row r="25" spans="1:10">
+      <c r="A25" s="4"/>
+      <c r="B25" s="21">
+        <v>21</v>
+      </c>
+      <c r="C25" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="D25" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="E25" s="24"/>
+      <c r="F25" s="24"/>
+      <c r="G25" s="24"/>
+      <c r="H25" s="24"/>
+      <c r="I25" s="24"/>
+      <c r="J25" s="24"/>
+    </row>
+    <row r="26" spans="1:10">
+      <c r="A26" s="4"/>
+      <c r="B26" s="21">
+        <v>22</v>
+      </c>
+      <c r="C26" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="D26" s="31" t="s">
+        <v>90</v>
+      </c>
+      <c r="E26" s="31" t="s">
+        <v>9</v>
+      </c>
+      <c r="F26" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="G26" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="H26" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="I26" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="J26" s="33" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10">
+      <c r="A27" s="4"/>
+      <c r="B27" s="21">
+        <v>23</v>
+      </c>
+      <c r="C27" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="D27" s="30"/>
+      <c r="E27" s="30"/>
+      <c r="F27" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="G27" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="H27" s="21"/>
+      <c r="I27" s="28"/>
+      <c r="J27" s="34"/>
+    </row>
+    <row r="28" spans="1:10">
+      <c r="A28" s="4"/>
+      <c r="B28" s="21">
+        <v>24</v>
+      </c>
+      <c r="C28" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="D28" s="30"/>
+      <c r="E28" s="30"/>
+      <c r="F28" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="G28" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="H28" s="21"/>
+      <c r="I28" s="28"/>
+      <c r="J28" s="34"/>
+    </row>
+    <row r="29" spans="1:10">
+      <c r="A29" s="4"/>
+      <c r="B29" s="21">
+        <v>25</v>
+      </c>
+      <c r="C29" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="D29" s="30"/>
+      <c r="E29" s="30"/>
+      <c r="F29" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="G29" s="21"/>
+      <c r="H29" s="21"/>
+      <c r="I29" s="28"/>
+      <c r="J29" s="34"/>
+    </row>
+    <row r="30" spans="1:10">
+      <c r="A30" s="4"/>
+      <c r="B30" s="21">
+        <v>26</v>
+      </c>
+      <c r="C30" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="D30" s="30"/>
+      <c r="E30" s="30"/>
+      <c r="F30" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="G30" s="21"/>
+      <c r="H30" s="21"/>
+      <c r="I30" s="28"/>
+      <c r="J30" s="35"/>
+    </row>
+    <row r="31" spans="1:10">
+      <c r="A31" s="4"/>
+      <c r="B31" s="21">
+        <v>27</v>
+      </c>
+      <c r="C31" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="D31" s="30"/>
+      <c r="E31" s="30"/>
+      <c r="F31" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="G31" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="H31" s="21"/>
+      <c r="I31" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="J31" s="50" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10">
+      <c r="A32" s="4"/>
+      <c r="B32" s="21">
+        <v>28</v>
+      </c>
+      <c r="C32" s="21" t="s">
+        <v>75</v>
+      </c>
+      <c r="D32" s="30"/>
+      <c r="E32" s="30"/>
+      <c r="F32" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="G32" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="H32" s="21"/>
+      <c r="I32" s="28"/>
+      <c r="J32" s="50"/>
+    </row>
+    <row r="33" spans="1:10">
+      <c r="A33" s="4"/>
+      <c r="B33" s="21">
+        <v>29</v>
+      </c>
+      <c r="C33" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="D33" s="47" t="s">
+        <v>79</v>
+      </c>
+      <c r="E33" s="48"/>
+      <c r="F33" s="48"/>
+      <c r="G33" s="48"/>
+      <c r="H33" s="48"/>
+      <c r="I33" s="48"/>
+      <c r="J33" s="49"/>
+    </row>
+    <row r="34" spans="1:10">
+      <c r="A34" s="4"/>
+      <c r="B34" s="21">
+        <v>30</v>
+      </c>
+      <c r="C34" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="D34" s="31" t="s">
+        <v>90</v>
+      </c>
+      <c r="E34" s="31" t="s">
+        <v>9</v>
+      </c>
+      <c r="F34" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="G34" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="H34" s="21"/>
+      <c r="I34" s="28" t="s">
+        <v>102</v>
+      </c>
+      <c r="J34" s="36" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10">
+      <c r="A35" s="4"/>
+      <c r="B35" s="21">
+        <v>31</v>
+      </c>
+      <c r="C35" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="D35" s="30"/>
+      <c r="E35" s="30"/>
+      <c r="F35" s="21" t="s">
+        <v>84</v>
+      </c>
+      <c r="G35" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="H35" s="21"/>
+      <c r="I35" s="28"/>
+      <c r="J35" s="36"/>
+    </row>
+    <row r="36" spans="1:10">
+      <c r="A36" s="4"/>
+      <c r="B36" s="21">
+        <v>32</v>
+      </c>
+      <c r="C36" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D36" s="30"/>
+      <c r="E36" s="30"/>
+      <c r="F36" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="G36" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="H36" s="21"/>
+      <c r="I36" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="J36" s="9" t="s">
+        <v>146</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="33">
+    <mergeCell ref="D33:J33"/>
+    <mergeCell ref="D34:D36"/>
+    <mergeCell ref="E34:E36"/>
+    <mergeCell ref="I34:I35"/>
+    <mergeCell ref="J34:J35"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="D22:J22"/>
+    <mergeCell ref="D24:J24"/>
+    <mergeCell ref="D25:J25"/>
+    <mergeCell ref="D26:D32"/>
+    <mergeCell ref="E26:E32"/>
+    <mergeCell ref="I26:I30"/>
+    <mergeCell ref="J26:J30"/>
+    <mergeCell ref="I31:I32"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="D13:D21"/>
+    <mergeCell ref="E13:E21"/>
+    <mergeCell ref="I14:I18"/>
+    <mergeCell ref="J14:J18"/>
+    <mergeCell ref="I19:I21"/>
+    <mergeCell ref="J19:J21"/>
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="D8:J9"/>
+    <mergeCell ref="E10:E12"/>
+    <mergeCell ref="I10:I12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="J3:J4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="B2:M36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1218,17 +2082,17 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:13">
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="37" t="s">
         <v>106</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
+      <c r="G2" s="37"/>
+      <c r="H2" s="37"/>
+      <c r="I2" s="37"/>
+      <c r="J2" s="37"/>
       <c r="L2" s="2" t="s">
         <v>108</v>
       </c>
@@ -1237,25 +2101,25 @@
       </c>
     </row>
     <row r="3" spans="2:13">
-      <c r="B3" s="45" t="s">
+      <c r="B3" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="45" t="s">
+      <c r="C3" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="45" t="s">
+      <c r="D3" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="50" t="s">
+      <c r="E3" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="50"/>
-      <c r="G3" s="50"/>
-      <c r="H3" s="50"/>
-      <c r="I3" s="23" t="s">
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="29" t="s">
         <v>92</v>
       </c>
-      <c r="J3" s="23" t="s">
+      <c r="J3" s="29" t="s">
         <v>103</v>
       </c>
       <c r="L3" s="2" t="s">
@@ -1266,9 +2130,9 @@
       </c>
     </row>
     <row r="4" spans="2:13">
-      <c r="B4" s="45"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
       <c r="E4" s="3" t="s">
         <v>3</v>
       </c>
@@ -1281,8 +2145,8 @@
       <c r="H4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I4" s="23"/>
-      <c r="J4" s="23"/>
+      <c r="I4" s="29"/>
+      <c r="J4" s="29"/>
       <c r="L4" s="2" t="s">
         <v>110</v>
       </c>
@@ -1298,7 +2162,7 @@
       <c r="C5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="43" t="s">
+      <c r="D5" s="31" t="s">
         <v>90</v>
       </c>
       <c r="E5" s="6" t="s">
@@ -1325,7 +2189,7 @@
       <c r="C6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="44"/>
+      <c r="D6" s="30"/>
       <c r="E6" s="6" t="s">
         <v>9</v>
       </c>
@@ -1348,7 +2212,7 @@
       <c r="C7" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="44"/>
+      <c r="D7" s="30"/>
       <c r="E7" s="6" t="s">
         <v>9</v>
       </c>
@@ -1375,15 +2239,15 @@
       <c r="C8" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="25" t="s">
+      <c r="D8" s="38" t="s">
         <v>89</v>
       </c>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26"/>
-      <c r="J8" s="27"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="39"/>
+      <c r="I8" s="39"/>
+      <c r="J8" s="40"/>
     </row>
     <row r="9" spans="2:13">
       <c r="B9" s="6">
@@ -1392,13 +2256,13 @@
       <c r="C9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="28"/>
-      <c r="E9" s="29"/>
-      <c r="F9" s="29"/>
-      <c r="G9" s="29"/>
-      <c r="H9" s="29"/>
-      <c r="I9" s="29"/>
-      <c r="J9" s="30"/>
+      <c r="D9" s="41"/>
+      <c r="E9" s="42"/>
+      <c r="F9" s="42"/>
+      <c r="G9" s="42"/>
+      <c r="H9" s="42"/>
+      <c r="I9" s="42"/>
+      <c r="J9" s="43"/>
     </row>
     <row r="10" spans="2:13">
       <c r="B10" s="6">
@@ -1410,7 +2274,7 @@
       <c r="D10" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E10" s="44" t="s">
+      <c r="E10" s="30" t="s">
         <v>9</v>
       </c>
       <c r="F10" s="6" t="s">
@@ -1420,10 +2284,10 @@
         <v>22</v>
       </c>
       <c r="H10" s="6"/>
-      <c r="I10" s="42" t="s">
+      <c r="I10" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="J10" s="39" t="s">
+      <c r="J10" s="52" t="s">
         <v>111</v>
       </c>
     </row>
@@ -1434,17 +2298,17 @@
       <c r="C11" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="43" t="s">
+      <c r="D11" s="31" t="s">
         <v>91</v>
       </c>
-      <c r="E11" s="44"/>
+      <c r="E11" s="30"/>
       <c r="F11" s="6" t="s">
         <v>24</v>
       </c>
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
-      <c r="I11" s="42"/>
-      <c r="J11" s="40"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="53"/>
     </row>
     <row r="12" spans="2:13">
       <c r="B12" s="6">
@@ -1453,15 +2317,15 @@
       <c r="C12" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="44"/>
-      <c r="E12" s="44"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="30"/>
       <c r="F12" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
-      <c r="I12" s="42"/>
-      <c r="J12" s="41"/>
+      <c r="I12" s="28"/>
+      <c r="J12" s="54"/>
     </row>
     <row r="13" spans="2:13">
       <c r="B13" s="6">
@@ -1470,10 +2334,10 @@
       <c r="C13" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D13" s="43" t="s">
+      <c r="D13" s="31" t="s">
         <v>90</v>
       </c>
-      <c r="E13" s="44" t="s">
+      <c r="E13" s="30" t="s">
         <v>9</v>
       </c>
       <c r="F13" s="6" t="s">
@@ -1495,8 +2359,8 @@
       <c r="C14" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D14" s="44"/>
-      <c r="E14" s="44"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="30"/>
       <c r="F14" s="6" t="s">
         <v>30</v>
       </c>
@@ -1504,10 +2368,10 @@
         <v>31</v>
       </c>
       <c r="H14" s="6"/>
-      <c r="I14" s="42" t="s">
+      <c r="I14" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="J14" s="19" t="s">
+      <c r="J14" s="33" t="s">
         <v>104</v>
       </c>
     </row>
@@ -1518,15 +2382,15 @@
       <c r="C15" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="44"/>
-      <c r="E15" s="44"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="30"/>
       <c r="F15" s="6" t="s">
         <v>33</v>
       </c>
       <c r="G15" s="6"/>
       <c r="H15" s="6"/>
-      <c r="I15" s="42"/>
-      <c r="J15" s="20"/>
+      <c r="I15" s="28"/>
+      <c r="J15" s="34"/>
     </row>
     <row r="16" spans="2:13">
       <c r="B16" s="6">
@@ -1535,8 +2399,8 @@
       <c r="C16" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="44"/>
-      <c r="E16" s="44"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="30"/>
       <c r="F16" s="6" t="s">
         <v>35</v>
       </c>
@@ -1544,8 +2408,8 @@
         <v>36</v>
       </c>
       <c r="H16" s="6"/>
-      <c r="I16" s="42"/>
-      <c r="J16" s="20"/>
+      <c r="I16" s="28"/>
+      <c r="J16" s="34"/>
     </row>
     <row r="17" spans="2:10">
       <c r="B17" s="6">
@@ -1554,15 +2418,15 @@
       <c r="C17" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D17" s="44"/>
-      <c r="E17" s="44"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="30"/>
       <c r="F17" s="6" t="s">
         <v>38</v>
       </c>
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
-      <c r="I17" s="42"/>
-      <c r="J17" s="20"/>
+      <c r="I17" s="28"/>
+      <c r="J17" s="34"/>
     </row>
     <row r="18" spans="2:10">
       <c r="B18" s="6">
@@ -1571,8 +2435,8 @@
       <c r="C18" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D18" s="44"/>
-      <c r="E18" s="44"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="30"/>
       <c r="F18" s="6" t="s">
         <v>40</v>
       </c>
@@ -1580,8 +2444,8 @@
         <v>45</v>
       </c>
       <c r="H18" s="6"/>
-      <c r="I18" s="42"/>
-      <c r="J18" s="21"/>
+      <c r="I18" s="28"/>
+      <c r="J18" s="35"/>
     </row>
     <row r="19" spans="2:10">
       <c r="B19" s="6">
@@ -1590,8 +2454,8 @@
       <c r="C19" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D19" s="44"/>
-      <c r="E19" s="44"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
       <c r="F19" s="6" t="s">
         <v>42</v>
       </c>
@@ -1601,10 +2465,10 @@
       <c r="H19" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="I19" s="42" t="s">
+      <c r="I19" s="28" t="s">
         <v>99</v>
       </c>
-      <c r="J19" s="38" t="s">
+      <c r="J19" s="51" t="s">
         <v>94</v>
       </c>
     </row>
@@ -1615,8 +2479,8 @@
       <c r="C20" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="D20" s="44"/>
-      <c r="E20" s="44"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="30"/>
       <c r="F20" s="6" t="s">
         <v>47</v>
       </c>
@@ -1624,8 +2488,8 @@
         <v>48</v>
       </c>
       <c r="H20" s="6"/>
-      <c r="I20" s="42"/>
-      <c r="J20" s="38"/>
+      <c r="I20" s="28"/>
+      <c r="J20" s="51"/>
     </row>
     <row r="21" spans="2:10">
       <c r="B21" s="6">
@@ -1634,8 +2498,8 @@
       <c r="C21" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="D21" s="44"/>
-      <c r="E21" s="44"/>
+      <c r="D21" s="30"/>
+      <c r="E21" s="30"/>
       <c r="F21" s="6" t="s">
         <v>50</v>
       </c>
@@ -1643,8 +2507,8 @@
         <v>51</v>
       </c>
       <c r="H21" s="6"/>
-      <c r="I21" s="42"/>
-      <c r="J21" s="38"/>
+      <c r="I21" s="28"/>
+      <c r="J21" s="51"/>
     </row>
     <row r="22" spans="2:10">
       <c r="B22" s="6">
@@ -1653,15 +2517,15 @@
       <c r="C22" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D22" s="31" t="s">
+      <c r="D22" s="44" t="s">
         <v>89</v>
       </c>
-      <c r="E22" s="32"/>
-      <c r="F22" s="32"/>
-      <c r="G22" s="32"/>
-      <c r="H22" s="32"/>
-      <c r="I22" s="32"/>
-      <c r="J22" s="33"/>
+      <c r="E22" s="45"/>
+      <c r="F22" s="45"/>
+      <c r="G22" s="45"/>
+      <c r="H22" s="45"/>
+      <c r="I22" s="45"/>
+      <c r="J22" s="46"/>
     </row>
     <row r="23" spans="2:10">
       <c r="B23" s="6">
@@ -1699,15 +2563,15 @@
       <c r="C24" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D24" s="47" t="s">
+      <c r="D24" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="E24" s="48"/>
-      <c r="F24" s="48"/>
-      <c r="G24" s="48"/>
-      <c r="H24" s="48"/>
-      <c r="I24" s="48"/>
-      <c r="J24" s="49"/>
+      <c r="E24" s="26"/>
+      <c r="F24" s="26"/>
+      <c r="G24" s="26"/>
+      <c r="H24" s="26"/>
+      <c r="I24" s="26"/>
+      <c r="J24" s="27"/>
     </row>
     <row r="25" spans="2:10">
       <c r="B25" s="6">
@@ -1716,15 +2580,15 @@
       <c r="C25" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D25" s="46" t="s">
+      <c r="D25" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="E25" s="46"/>
-      <c r="F25" s="46"/>
-      <c r="G25" s="46"/>
-      <c r="H25" s="46"/>
-      <c r="I25" s="46"/>
-      <c r="J25" s="46"/>
+      <c r="E25" s="24"/>
+      <c r="F25" s="24"/>
+      <c r="G25" s="24"/>
+      <c r="H25" s="24"/>
+      <c r="I25" s="24"/>
+      <c r="J25" s="24"/>
     </row>
     <row r="26" spans="2:10">
       <c r="B26" s="6">
@@ -1733,10 +2597,10 @@
       <c r="C26" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="D26" s="43" t="s">
+      <c r="D26" s="31" t="s">
         <v>90</v>
       </c>
-      <c r="E26" s="43" t="s">
+      <c r="E26" s="31" t="s">
         <v>9</v>
       </c>
       <c r="F26" s="6" t="s">
@@ -1748,10 +2612,10 @@
       <c r="H26" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="I26" s="42" t="s">
+      <c r="I26" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="J26" s="19" t="s">
+      <c r="J26" s="33" t="s">
         <v>104</v>
       </c>
     </row>
@@ -1762,8 +2626,8 @@
       <c r="C27" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D27" s="44"/>
-      <c r="E27" s="44"/>
+      <c r="D27" s="30"/>
+      <c r="E27" s="30"/>
       <c r="F27" s="6" t="s">
         <v>63</v>
       </c>
@@ -1771,8 +2635,8 @@
         <v>64</v>
       </c>
       <c r="H27" s="6"/>
-      <c r="I27" s="42"/>
-      <c r="J27" s="20"/>
+      <c r="I27" s="28"/>
+      <c r="J27" s="34"/>
     </row>
     <row r="28" spans="2:10">
       <c r="B28" s="6">
@@ -1781,8 +2645,8 @@
       <c r="C28" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="D28" s="44"/>
-      <c r="E28" s="44"/>
+      <c r="D28" s="30"/>
+      <c r="E28" s="30"/>
       <c r="F28" s="6" t="s">
         <v>66</v>
       </c>
@@ -1790,8 +2654,8 @@
         <v>67</v>
       </c>
       <c r="H28" s="6"/>
-      <c r="I28" s="42"/>
-      <c r="J28" s="20"/>
+      <c r="I28" s="28"/>
+      <c r="J28" s="34"/>
     </row>
     <row r="29" spans="2:10">
       <c r="B29" s="6">
@@ -1800,15 +2664,15 @@
       <c r="C29" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="D29" s="44"/>
-      <c r="E29" s="44"/>
+      <c r="D29" s="30"/>
+      <c r="E29" s="30"/>
       <c r="F29" s="6" t="s">
         <v>69</v>
       </c>
       <c r="G29" s="6"/>
       <c r="H29" s="6"/>
-      <c r="I29" s="42"/>
-      <c r="J29" s="20"/>
+      <c r="I29" s="28"/>
+      <c r="J29" s="34"/>
     </row>
     <row r="30" spans="2:10">
       <c r="B30" s="6">
@@ -1817,15 +2681,15 @@
       <c r="C30" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D30" s="44"/>
-      <c r="E30" s="44"/>
+      <c r="D30" s="30"/>
+      <c r="E30" s="30"/>
       <c r="F30" s="6" t="s">
         <v>71</v>
       </c>
       <c r="G30" s="6"/>
       <c r="H30" s="6"/>
-      <c r="I30" s="42"/>
-      <c r="J30" s="21"/>
+      <c r="I30" s="28"/>
+      <c r="J30" s="35"/>
     </row>
     <row r="31" spans="2:10">
       <c r="B31" s="6">
@@ -1834,8 +2698,8 @@
       <c r="C31" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="D31" s="44"/>
-      <c r="E31" s="44"/>
+      <c r="D31" s="30"/>
+      <c r="E31" s="30"/>
       <c r="F31" s="6" t="s">
         <v>73</v>
       </c>
@@ -1843,10 +2707,10 @@
         <v>74</v>
       </c>
       <c r="H31" s="6"/>
-      <c r="I31" s="42" t="s">
+      <c r="I31" s="28" t="s">
         <v>97</v>
       </c>
-      <c r="J31" s="37" t="s">
+      <c r="J31" s="50" t="s">
         <v>96</v>
       </c>
     </row>
@@ -1857,8 +2721,8 @@
       <c r="C32" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="D32" s="44"/>
-      <c r="E32" s="44"/>
+      <c r="D32" s="30"/>
+      <c r="E32" s="30"/>
       <c r="F32" s="6" t="s">
         <v>76</v>
       </c>
@@ -1866,8 +2730,8 @@
         <v>77</v>
       </c>
       <c r="H32" s="6"/>
-      <c r="I32" s="42"/>
-      <c r="J32" s="37"/>
+      <c r="I32" s="28"/>
+      <c r="J32" s="50"/>
     </row>
     <row r="33" spans="2:10">
       <c r="B33" s="6">
@@ -1876,15 +2740,15 @@
       <c r="C33" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="D33" s="34" t="s">
+      <c r="D33" s="47" t="s">
         <v>79</v>
       </c>
-      <c r="E33" s="35"/>
-      <c r="F33" s="35"/>
-      <c r="G33" s="35"/>
-      <c r="H33" s="35"/>
-      <c r="I33" s="35"/>
-      <c r="J33" s="36"/>
+      <c r="E33" s="48"/>
+      <c r="F33" s="48"/>
+      <c r="G33" s="48"/>
+      <c r="H33" s="48"/>
+      <c r="I33" s="48"/>
+      <c r="J33" s="49"/>
     </row>
     <row r="34" spans="2:10" ht="15" customHeight="1">
       <c r="B34" s="6">
@@ -1893,10 +2757,10 @@
       <c r="C34" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="D34" s="43" t="s">
+      <c r="D34" s="31" t="s">
         <v>90</v>
       </c>
-      <c r="E34" s="43" t="s">
+      <c r="E34" s="31" t="s">
         <v>9</v>
       </c>
       <c r="F34" s="6" t="s">
@@ -1906,10 +2770,10 @@
         <v>82</v>
       </c>
       <c r="H34" s="6"/>
-      <c r="I34" s="42" t="s">
+      <c r="I34" s="28" t="s">
         <v>102</v>
       </c>
-      <c r="J34" s="22" t="s">
+      <c r="J34" s="36" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1920,8 +2784,8 @@
       <c r="C35" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="D35" s="44"/>
-      <c r="E35" s="44"/>
+      <c r="D35" s="30"/>
+      <c r="E35" s="30"/>
       <c r="F35" s="6" t="s">
         <v>84</v>
       </c>
@@ -1929,8 +2793,8 @@
         <v>85</v>
       </c>
       <c r="H35" s="6"/>
-      <c r="I35" s="42"/>
-      <c r="J35" s="22"/>
+      <c r="I35" s="28"/>
+      <c r="J35" s="36"/>
     </row>
     <row r="36" spans="2:10">
       <c r="B36" s="6">
@@ -1939,8 +2803,8 @@
       <c r="C36" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="D36" s="44"/>
-      <c r="E36" s="44"/>
+      <c r="D36" s="30"/>
+      <c r="E36" s="30"/>
       <c r="F36" s="6" t="s">
         <v>87</v>
       </c>
@@ -1957,23 +2821,6 @@
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="D25:J25"/>
-    <mergeCell ref="D24:J24"/>
-    <mergeCell ref="I10:I12"/>
-    <mergeCell ref="I3:I4"/>
-    <mergeCell ref="E10:E12"/>
-    <mergeCell ref="D5:D7"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E3:H3"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="D34:D36"/>
-    <mergeCell ref="E13:E21"/>
-    <mergeCell ref="E26:E32"/>
-    <mergeCell ref="E34:E36"/>
-    <mergeCell ref="D13:D21"/>
-    <mergeCell ref="D26:D32"/>
     <mergeCell ref="J26:J30"/>
     <mergeCell ref="J34:J35"/>
     <mergeCell ref="J3:J4"/>
@@ -1990,13 +2837,30 @@
     <mergeCell ref="I26:I30"/>
     <mergeCell ref="I14:I18"/>
     <mergeCell ref="I31:I32"/>
+    <mergeCell ref="D34:D36"/>
+    <mergeCell ref="E13:E21"/>
+    <mergeCell ref="E26:E32"/>
+    <mergeCell ref="E34:E36"/>
+    <mergeCell ref="D13:D21"/>
+    <mergeCell ref="D26:D32"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="D25:J25"/>
+    <mergeCell ref="D24:J24"/>
+    <mergeCell ref="I10:I12"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="E10:E12"/>
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="D3:D4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967294" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="B2:H39"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2010,15 +2874,15 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8">
-      <c r="B2" s="51" t="s">
+      <c r="B2" s="55" t="s">
         <v>117</v>
       </c>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
-      <c r="H2" s="53"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="57"/>
     </row>
     <row r="3" spans="2:8">
       <c r="B3" s="16" t="s">

</xml_diff>

<commit_message>
added V1.0 BOM, updated greber
</commit_message>
<xml_diff>
--- a/Design/HLD_Design/Project_OAK_MCU_Pinouts.xlsx
+++ b/Design/HLD_Design/Project_OAK_MCU_Pinouts.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="152">
   <si>
     <t>S. No</t>
   </si>
@@ -351,12 +351,6 @@
     <t>Used GPIOs:</t>
   </si>
   <si>
-    <t>Excess GPIOs:</t>
-  </si>
-  <si>
-    <t>Future use</t>
-  </si>
-  <si>
     <t>ANALOG POWER</t>
   </si>
   <si>
@@ -462,9 +456,6 @@
     <t>RTC + ACC</t>
   </si>
   <si>
-    <t>ACC_INT1/2</t>
-  </si>
-  <si>
     <t>PWR_BTN</t>
   </si>
   <si>
@@ -472,6 +463,18 @@
   </si>
   <si>
     <t>DWN_BTN</t>
+  </si>
+  <si>
+    <t>ACTIVITY LED</t>
+  </si>
+  <si>
+    <t>ACC_INT1</t>
+  </si>
+  <si>
+    <t>BAT VOL MON / ACC_INT2</t>
+  </si>
+  <si>
+    <t>Balance GPIOs:</t>
   </si>
 </sst>
 </file>
@@ -606,7 +609,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -765,11 +768,28 @@
       </bottom>
       <diagonal/>
     </border>
+    <border diagonalUp="1" diagonalDown="1">
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal style="thin">
+        <color indexed="64"/>
+      </diagonal>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -840,6 +860,84 @@
     <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -852,90 +950,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -943,6 +957,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1257,17 +1274,17 @@
   <sheetData>
     <row r="2" spans="1:13">
       <c r="A2" s="4"/>
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="50" t="s">
         <v>106</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="H2" s="50"/>
+      <c r="I2" s="50"/>
+      <c r="J2" s="50"/>
       <c r="L2" s="2" t="s">
         <v>108</v>
       </c>
@@ -1277,25 +1294,25 @@
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="4"/>
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="C3" s="51" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="25" t="s">
+      <c r="D3" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="26" t="s">
+      <c r="E3" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="26"/>
-      <c r="G3" s="26"/>
-      <c r="H3" s="26"/>
-      <c r="I3" s="27" t="s">
+      <c r="F3" s="52"/>
+      <c r="G3" s="52"/>
+      <c r="H3" s="52"/>
+      <c r="I3" s="53" t="s">
         <v>92</v>
       </c>
-      <c r="J3" s="27" t="s">
+      <c r="J3" s="53" t="s">
         <v>103</v>
       </c>
       <c r="L3" s="2" t="s">
@@ -1307,9 +1324,9 @@
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="4"/>
-      <c r="B4" s="25"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
+      <c r="B4" s="51"/>
+      <c r="C4" s="51"/>
+      <c r="D4" s="51"/>
       <c r="E4" s="22" t="s">
         <v>3</v>
       </c>
@@ -1322,10 +1339,10 @@
       <c r="H4" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="I4" s="27"/>
-      <c r="J4" s="27"/>
+      <c r="I4" s="53"/>
+      <c r="J4" s="53"/>
       <c r="L4" s="2" t="s">
-        <v>110</v>
+        <v>151</v>
       </c>
       <c r="M4" s="2">
         <f>M2-M3</f>
@@ -1381,7 +1398,7 @@
         <v>100</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1409,7 +1426,7 @@
         <v>9</v>
       </c>
       <c r="J7" s="12" t="s">
-        <v>107</v>
+        <v>148</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -1420,15 +1437,15 @@
       <c r="C8" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="30" t="s">
+      <c r="D8" s="44" t="s">
         <v>89</v>
       </c>
-      <c r="E8" s="31"/>
-      <c r="F8" s="31"/>
-      <c r="G8" s="31"/>
-      <c r="H8" s="31"/>
-      <c r="I8" s="31"/>
-      <c r="J8" s="32"/>
+      <c r="E8" s="45"/>
+      <c r="F8" s="45"/>
+      <c r="G8" s="45"/>
+      <c r="H8" s="45"/>
+      <c r="I8" s="45"/>
+      <c r="J8" s="46"/>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="4"/>
@@ -1438,13 +1455,13 @@
       <c r="C9" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="33"/>
-      <c r="E9" s="34"/>
-      <c r="F9" s="34"/>
-      <c r="G9" s="34"/>
-      <c r="H9" s="34"/>
-      <c r="I9" s="34"/>
-      <c r="J9" s="35"/>
+      <c r="D9" s="47"/>
+      <c r="E9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="48"/>
+      <c r="H9" s="48"/>
+      <c r="I9" s="48"/>
+      <c r="J9" s="49"/>
     </row>
     <row r="10" spans="1:13">
       <c r="A10" s="4"/>
@@ -1467,11 +1484,11 @@
         <v>22</v>
       </c>
       <c r="H10" s="21"/>
-      <c r="I10" s="36" t="s">
+      <c r="I10" s="30" t="s">
         <v>9</v>
       </c>
       <c r="J10" s="23" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1491,10 +1508,8 @@
       </c>
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
-      <c r="I11" s="36"/>
-      <c r="J11" s="28" t="s">
-        <v>111</v>
-      </c>
+      <c r="I11" s="30"/>
+      <c r="J11" s="57"/>
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="4"/>
@@ -1511,8 +1526,8 @@
       </c>
       <c r="G12" s="21"/>
       <c r="H12" s="21"/>
-      <c r="I12" s="36"/>
-      <c r="J12" s="28"/>
+      <c r="I12" s="30"/>
+      <c r="J12" s="57"/>
     </row>
     <row r="13" spans="1:13">
       <c r="A13" s="4"/>
@@ -1537,7 +1552,7 @@
         <v>100</v>
       </c>
       <c r="J13" s="9" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="14" spans="1:13">
@@ -1557,10 +1572,10 @@
         <v>31</v>
       </c>
       <c r="H14" s="21"/>
-      <c r="I14" s="36" t="s">
+      <c r="I14" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="J14" s="44" t="s">
+      <c r="J14" s="32" t="s">
         <v>104</v>
       </c>
     </row>
@@ -1579,8 +1594,8 @@
       </c>
       <c r="G15" s="21"/>
       <c r="H15" s="21"/>
-      <c r="I15" s="36"/>
-      <c r="J15" s="45"/>
+      <c r="I15" s="30"/>
+      <c r="J15" s="33"/>
     </row>
     <row r="16" spans="1:13">
       <c r="A16" s="4"/>
@@ -1599,8 +1614,8 @@
         <v>36</v>
       </c>
       <c r="H16" s="21"/>
-      <c r="I16" s="36"/>
-      <c r="J16" s="45"/>
+      <c r="I16" s="30"/>
+      <c r="J16" s="33"/>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="4"/>
@@ -1617,8 +1632,8 @@
       </c>
       <c r="G17" s="21"/>
       <c r="H17" s="21"/>
-      <c r="I17" s="36"/>
-      <c r="J17" s="45"/>
+      <c r="I17" s="30"/>
+      <c r="J17" s="33"/>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="4"/>
@@ -1637,8 +1652,8 @@
         <v>45</v>
       </c>
       <c r="H18" s="21"/>
-      <c r="I18" s="36"/>
-      <c r="J18" s="46"/>
+      <c r="I18" s="30"/>
+      <c r="J18" s="34"/>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="4"/>
@@ -1659,10 +1674,10 @@
       <c r="H19" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="I19" s="36" t="s">
+      <c r="I19" s="30" t="s">
         <v>99</v>
       </c>
-      <c r="J19" s="48" t="s">
+      <c r="J19" s="35" t="s">
         <v>94</v>
       </c>
     </row>
@@ -1683,8 +1698,8 @@
         <v>48</v>
       </c>
       <c r="H20" s="21"/>
-      <c r="I20" s="36"/>
-      <c r="J20" s="48"/>
+      <c r="I20" s="30"/>
+      <c r="J20" s="35"/>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="4"/>
@@ -1703,8 +1718,8 @@
         <v>51</v>
       </c>
       <c r="H21" s="21"/>
-      <c r="I21" s="36"/>
-      <c r="J21" s="48"/>
+      <c r="I21" s="30"/>
+      <c r="J21" s="35"/>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="4"/>
@@ -1714,15 +1729,15 @@
       <c r="C22" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="D22" s="37" t="s">
+      <c r="D22" s="36" t="s">
         <v>89</v>
       </c>
-      <c r="E22" s="38"/>
-      <c r="F22" s="38"/>
-      <c r="G22" s="38"/>
-      <c r="H22" s="38"/>
-      <c r="I22" s="38"/>
-      <c r="J22" s="39"/>
+      <c r="E22" s="37"/>
+      <c r="F22" s="37"/>
+      <c r="G22" s="37"/>
+      <c r="H22" s="37"/>
+      <c r="I22" s="37"/>
+      <c r="J22" s="38"/>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="4"/>
@@ -1750,8 +1765,8 @@
       <c r="I23" s="19" t="s">
         <v>98</v>
       </c>
-      <c r="J23" s="19" t="s">
-        <v>95</v>
+      <c r="J23" s="24" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -1762,15 +1777,15 @@
       <c r="C24" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="D24" s="40" t="s">
-        <v>112</v>
-      </c>
-      <c r="E24" s="41"/>
-      <c r="F24" s="41"/>
-      <c r="G24" s="41"/>
-      <c r="H24" s="41"/>
-      <c r="I24" s="41"/>
-      <c r="J24" s="42"/>
+      <c r="D24" s="39" t="s">
+        <v>110</v>
+      </c>
+      <c r="E24" s="40"/>
+      <c r="F24" s="40"/>
+      <c r="G24" s="40"/>
+      <c r="H24" s="40"/>
+      <c r="I24" s="40"/>
+      <c r="J24" s="41"/>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="4"/>
@@ -1780,15 +1795,15 @@
       <c r="C25" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="D25" s="43" t="s">
+      <c r="D25" s="42" t="s">
         <v>89</v>
       </c>
-      <c r="E25" s="43"/>
-      <c r="F25" s="43"/>
-      <c r="G25" s="43"/>
-      <c r="H25" s="43"/>
-      <c r="I25" s="43"/>
-      <c r="J25" s="43"/>
+      <c r="E25" s="42"/>
+      <c r="F25" s="42"/>
+      <c r="G25" s="42"/>
+      <c r="H25" s="42"/>
+      <c r="I25" s="42"/>
+      <c r="J25" s="42"/>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="4"/>
@@ -1813,10 +1828,10 @@
       <c r="H26" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="I26" s="36" t="s">
+      <c r="I26" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="J26" s="44" t="s">
+      <c r="J26" s="32" t="s">
         <v>104</v>
       </c>
     </row>
@@ -1837,8 +1852,8 @@
         <v>64</v>
       </c>
       <c r="H27" s="21"/>
-      <c r="I27" s="36"/>
-      <c r="J27" s="45"/>
+      <c r="I27" s="30"/>
+      <c r="J27" s="33"/>
     </row>
     <row r="28" spans="1:10">
       <c r="A28" s="4"/>
@@ -1857,8 +1872,8 @@
         <v>67</v>
       </c>
       <c r="H28" s="21"/>
-      <c r="I28" s="36"/>
-      <c r="J28" s="45"/>
+      <c r="I28" s="30"/>
+      <c r="J28" s="33"/>
     </row>
     <row r="29" spans="1:10">
       <c r="A29" s="4"/>
@@ -1875,8 +1890,8 @@
       </c>
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
-      <c r="I29" s="36"/>
-      <c r="J29" s="45"/>
+      <c r="I29" s="30"/>
+      <c r="J29" s="33"/>
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="4"/>
@@ -1893,8 +1908,8 @@
       </c>
       <c r="G30" s="21"/>
       <c r="H30" s="21"/>
-      <c r="I30" s="36"/>
-      <c r="J30" s="46"/>
+      <c r="I30" s="30"/>
+      <c r="J30" s="34"/>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="4"/>
@@ -1913,11 +1928,11 @@
         <v>74</v>
       </c>
       <c r="H31" s="21"/>
-      <c r="I31" s="36" t="s">
+      <c r="I31" s="30" t="s">
         <v>97</v>
       </c>
-      <c r="J31" s="47" t="s">
-        <v>146</v>
+      <c r="J31" s="43" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -1937,8 +1952,8 @@
         <v>77</v>
       </c>
       <c r="H32" s="21"/>
-      <c r="I32" s="36"/>
-      <c r="J32" s="47"/>
+      <c r="I32" s="30"/>
+      <c r="J32" s="43"/>
     </row>
     <row r="33" spans="1:10">
       <c r="A33" s="4"/>
@@ -1948,15 +1963,15 @@
       <c r="C33" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="D33" s="49" t="s">
+      <c r="D33" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="E33" s="50"/>
-      <c r="F33" s="50"/>
-      <c r="G33" s="50"/>
-      <c r="H33" s="50"/>
-      <c r="I33" s="50"/>
-      <c r="J33" s="51"/>
+      <c r="E33" s="26"/>
+      <c r="F33" s="26"/>
+      <c r="G33" s="26"/>
+      <c r="H33" s="26"/>
+      <c r="I33" s="26"/>
+      <c r="J33" s="27"/>
     </row>
     <row r="34" spans="1:10">
       <c r="A34" s="4"/>
@@ -1979,11 +1994,11 @@
         <v>82</v>
       </c>
       <c r="H34" s="21"/>
-      <c r="I34" s="36" t="s">
+      <c r="I34" s="30" t="s">
         <v>102</v>
       </c>
-      <c r="J34" s="52" t="s">
-        <v>105</v>
+      <c r="J34" s="31" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="35" spans="1:10">
@@ -2003,8 +2018,8 @@
         <v>85</v>
       </c>
       <c r="H35" s="21"/>
-      <c r="I35" s="36"/>
-      <c r="J35" s="52"/>
+      <c r="I35" s="30"/>
+      <c r="J35" s="31"/>
     </row>
     <row r="36" spans="1:10">
       <c r="A36" s="4"/>
@@ -2027,7 +2042,7 @@
         <v>101</v>
       </c>
       <c r="J36" s="9" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -2037,17 +2052,19 @@
     <filterColumn colId="5" showButton="0"/>
   </autoFilter>
   <mergeCells count="33">
-    <mergeCell ref="D33:J33"/>
-    <mergeCell ref="D34:D36"/>
-    <mergeCell ref="E34:E36"/>
-    <mergeCell ref="I34:I35"/>
-    <mergeCell ref="J34:J35"/>
-    <mergeCell ref="D13:D21"/>
-    <mergeCell ref="E13:E21"/>
-    <mergeCell ref="I14:I18"/>
-    <mergeCell ref="J14:J18"/>
-    <mergeCell ref="I19:I21"/>
-    <mergeCell ref="J19:J21"/>
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="J3:J4"/>
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="D8:J9"/>
+    <mergeCell ref="E10:E12"/>
+    <mergeCell ref="I10:I12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="J11:J12"/>
     <mergeCell ref="D22:J22"/>
     <mergeCell ref="D24:J24"/>
     <mergeCell ref="D25:J25"/>
@@ -2057,21 +2074,20 @@
     <mergeCell ref="J26:J30"/>
     <mergeCell ref="I31:I32"/>
     <mergeCell ref="J31:J32"/>
-    <mergeCell ref="D5:D7"/>
-    <mergeCell ref="D8:J9"/>
-    <mergeCell ref="E10:E12"/>
-    <mergeCell ref="I10:I12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="B2:J2"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:H3"/>
-    <mergeCell ref="I3:I4"/>
-    <mergeCell ref="J3:J4"/>
+    <mergeCell ref="D13:D21"/>
+    <mergeCell ref="E13:E21"/>
+    <mergeCell ref="I14:I18"/>
+    <mergeCell ref="J14:J18"/>
+    <mergeCell ref="I19:I21"/>
+    <mergeCell ref="J19:J21"/>
+    <mergeCell ref="D33:J33"/>
+    <mergeCell ref="D34:D36"/>
+    <mergeCell ref="E34:E36"/>
+    <mergeCell ref="I34:I35"/>
+    <mergeCell ref="J34:J35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967294" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2096,17 +2112,17 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:13">
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="50" t="s">
         <v>106</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="H2" s="50"/>
+      <c r="I2" s="50"/>
+      <c r="J2" s="50"/>
       <c r="L2" s="2" t="s">
         <v>108</v>
       </c>
@@ -2115,25 +2131,25 @@
       </c>
     </row>
     <row r="3" spans="2:13">
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="C3" s="51" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="25" t="s">
+      <c r="D3" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="26" t="s">
+      <c r="E3" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="26"/>
-      <c r="G3" s="26"/>
-      <c r="H3" s="26"/>
-      <c r="I3" s="27" t="s">
+      <c r="F3" s="52"/>
+      <c r="G3" s="52"/>
+      <c r="H3" s="52"/>
+      <c r="I3" s="53" t="s">
         <v>92</v>
       </c>
-      <c r="J3" s="27" t="s">
+      <c r="J3" s="53" t="s">
         <v>103</v>
       </c>
       <c r="L3" s="2" t="s">
@@ -2144,9 +2160,9 @@
       </c>
     </row>
     <row r="4" spans="2:13">
-      <c r="B4" s="25"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
+      <c r="B4" s="51"/>
+      <c r="C4" s="51"/>
+      <c r="D4" s="51"/>
       <c r="E4" s="3" t="s">
         <v>3</v>
       </c>
@@ -2159,10 +2175,10 @@
       <c r="H4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I4" s="27"/>
-      <c r="J4" s="27"/>
+      <c r="I4" s="53"/>
+      <c r="J4" s="53"/>
       <c r="L4" s="2" t="s">
-        <v>110</v>
+        <v>151</v>
       </c>
       <c r="M4" s="2">
         <f>M2-M3</f>
@@ -2253,15 +2269,15 @@
       <c r="C8" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="30" t="s">
+      <c r="D8" s="44" t="s">
         <v>89</v>
       </c>
-      <c r="E8" s="31"/>
-      <c r="F8" s="31"/>
-      <c r="G8" s="31"/>
-      <c r="H8" s="31"/>
-      <c r="I8" s="31"/>
-      <c r="J8" s="32"/>
+      <c r="E8" s="45"/>
+      <c r="F8" s="45"/>
+      <c r="G8" s="45"/>
+      <c r="H8" s="45"/>
+      <c r="I8" s="45"/>
+      <c r="J8" s="46"/>
     </row>
     <row r="9" spans="2:13">
       <c r="B9" s="6">
@@ -2270,13 +2286,13 @@
       <c r="C9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="33"/>
-      <c r="E9" s="34"/>
-      <c r="F9" s="34"/>
-      <c r="G9" s="34"/>
-      <c r="H9" s="34"/>
-      <c r="I9" s="34"/>
-      <c r="J9" s="35"/>
+      <c r="D9" s="47"/>
+      <c r="E9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="48"/>
+      <c r="H9" s="48"/>
+      <c r="I9" s="48"/>
+      <c r="J9" s="49"/>
     </row>
     <row r="10" spans="2:13">
       <c r="B10" s="6">
@@ -2298,12 +2314,10 @@
         <v>22</v>
       </c>
       <c r="H10" s="6"/>
-      <c r="I10" s="36" t="s">
+      <c r="I10" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="J10" s="53" t="s">
-        <v>111</v>
-      </c>
+      <c r="J10" s="57"/>
     </row>
     <row r="11" spans="2:13">
       <c r="B11" s="6">
@@ -2321,8 +2335,8 @@
       </c>
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
-      <c r="I11" s="36"/>
-      <c r="J11" s="54"/>
+      <c r="I11" s="30"/>
+      <c r="J11" s="57"/>
     </row>
     <row r="12" spans="2:13">
       <c r="B12" s="6">
@@ -2338,8 +2352,8 @@
       </c>
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
-      <c r="I12" s="36"/>
-      <c r="J12" s="55"/>
+      <c r="I12" s="30"/>
+      <c r="J12" s="57"/>
     </row>
     <row r="13" spans="2:13">
       <c r="B13" s="6">
@@ -2382,10 +2396,10 @@
         <v>31</v>
       </c>
       <c r="H14" s="6"/>
-      <c r="I14" s="36" t="s">
+      <c r="I14" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="J14" s="44" t="s">
+      <c r="J14" s="32" t="s">
         <v>104</v>
       </c>
     </row>
@@ -2403,8 +2417,8 @@
       </c>
       <c r="G15" s="6"/>
       <c r="H15" s="6"/>
-      <c r="I15" s="36"/>
-      <c r="J15" s="45"/>
+      <c r="I15" s="30"/>
+      <c r="J15" s="33"/>
     </row>
     <row r="16" spans="2:13">
       <c r="B16" s="6">
@@ -2422,8 +2436,8 @@
         <v>36</v>
       </c>
       <c r="H16" s="6"/>
-      <c r="I16" s="36"/>
-      <c r="J16" s="45"/>
+      <c r="I16" s="30"/>
+      <c r="J16" s="33"/>
     </row>
     <row r="17" spans="2:10">
       <c r="B17" s="6">
@@ -2439,8 +2453,8 @@
       </c>
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
-      <c r="I17" s="36"/>
-      <c r="J17" s="45"/>
+      <c r="I17" s="30"/>
+      <c r="J17" s="33"/>
     </row>
     <row r="18" spans="2:10">
       <c r="B18" s="6">
@@ -2458,8 +2472,8 @@
         <v>45</v>
       </c>
       <c r="H18" s="6"/>
-      <c r="I18" s="36"/>
-      <c r="J18" s="46"/>
+      <c r="I18" s="30"/>
+      <c r="J18" s="34"/>
     </row>
     <row r="19" spans="2:10">
       <c r="B19" s="6">
@@ -2479,10 +2493,10 @@
       <c r="H19" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="I19" s="36" t="s">
+      <c r="I19" s="30" t="s">
         <v>99</v>
       </c>
-      <c r="J19" s="48" t="s">
+      <c r="J19" s="35" t="s">
         <v>94</v>
       </c>
     </row>
@@ -2502,8 +2516,8 @@
         <v>48</v>
       </c>
       <c r="H20" s="6"/>
-      <c r="I20" s="36"/>
-      <c r="J20" s="48"/>
+      <c r="I20" s="30"/>
+      <c r="J20" s="35"/>
     </row>
     <row r="21" spans="2:10">
       <c r="B21" s="6">
@@ -2521,8 +2535,8 @@
         <v>51</v>
       </c>
       <c r="H21" s="6"/>
-      <c r="I21" s="36"/>
-      <c r="J21" s="48"/>
+      <c r="I21" s="30"/>
+      <c r="J21" s="35"/>
     </row>
     <row r="22" spans="2:10">
       <c r="B22" s="6">
@@ -2531,15 +2545,15 @@
       <c r="C22" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D22" s="37" t="s">
+      <c r="D22" s="36" t="s">
         <v>89</v>
       </c>
-      <c r="E22" s="38"/>
-      <c r="F22" s="38"/>
-      <c r="G22" s="38"/>
-      <c r="H22" s="38"/>
-      <c r="I22" s="38"/>
-      <c r="J22" s="39"/>
+      <c r="E22" s="37"/>
+      <c r="F22" s="37"/>
+      <c r="G22" s="37"/>
+      <c r="H22" s="37"/>
+      <c r="I22" s="37"/>
+      <c r="J22" s="38"/>
     </row>
     <row r="23" spans="2:10">
       <c r="B23" s="6">
@@ -2577,15 +2591,15 @@
       <c r="C24" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D24" s="40" t="s">
-        <v>112</v>
-      </c>
-      <c r="E24" s="41"/>
-      <c r="F24" s="41"/>
-      <c r="G24" s="41"/>
-      <c r="H24" s="41"/>
-      <c r="I24" s="41"/>
-      <c r="J24" s="42"/>
+      <c r="D24" s="39" t="s">
+        <v>110</v>
+      </c>
+      <c r="E24" s="40"/>
+      <c r="F24" s="40"/>
+      <c r="G24" s="40"/>
+      <c r="H24" s="40"/>
+      <c r="I24" s="40"/>
+      <c r="J24" s="41"/>
     </row>
     <row r="25" spans="2:10">
       <c r="B25" s="6">
@@ -2594,15 +2608,15 @@
       <c r="C25" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D25" s="43" t="s">
+      <c r="D25" s="42" t="s">
         <v>89</v>
       </c>
-      <c r="E25" s="43"/>
-      <c r="F25" s="43"/>
-      <c r="G25" s="43"/>
-      <c r="H25" s="43"/>
-      <c r="I25" s="43"/>
-      <c r="J25" s="43"/>
+      <c r="E25" s="42"/>
+      <c r="F25" s="42"/>
+      <c r="G25" s="42"/>
+      <c r="H25" s="42"/>
+      <c r="I25" s="42"/>
+      <c r="J25" s="42"/>
     </row>
     <row r="26" spans="2:10">
       <c r="B26" s="6">
@@ -2626,10 +2640,10 @@
       <c r="H26" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="I26" s="36" t="s">
+      <c r="I26" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="J26" s="44" t="s">
+      <c r="J26" s="32" t="s">
         <v>104</v>
       </c>
     </row>
@@ -2649,8 +2663,8 @@
         <v>64</v>
       </c>
       <c r="H27" s="6"/>
-      <c r="I27" s="36"/>
-      <c r="J27" s="45"/>
+      <c r="I27" s="30"/>
+      <c r="J27" s="33"/>
     </row>
     <row r="28" spans="2:10">
       <c r="B28" s="6">
@@ -2668,8 +2682,8 @@
         <v>67</v>
       </c>
       <c r="H28" s="6"/>
-      <c r="I28" s="36"/>
-      <c r="J28" s="45"/>
+      <c r="I28" s="30"/>
+      <c r="J28" s="33"/>
     </row>
     <row r="29" spans="2:10">
       <c r="B29" s="6">
@@ -2685,8 +2699,8 @@
       </c>
       <c r="G29" s="6"/>
       <c r="H29" s="6"/>
-      <c r="I29" s="36"/>
-      <c r="J29" s="45"/>
+      <c r="I29" s="30"/>
+      <c r="J29" s="33"/>
     </row>
     <row r="30" spans="2:10">
       <c r="B30" s="6">
@@ -2702,8 +2716,8 @@
       </c>
       <c r="G30" s="6"/>
       <c r="H30" s="6"/>
-      <c r="I30" s="36"/>
-      <c r="J30" s="46"/>
+      <c r="I30" s="30"/>
+      <c r="J30" s="34"/>
     </row>
     <row r="31" spans="2:10">
       <c r="B31" s="6">
@@ -2721,10 +2735,10 @@
         <v>74</v>
       </c>
       <c r="H31" s="6"/>
-      <c r="I31" s="36" t="s">
+      <c r="I31" s="30" t="s">
         <v>97</v>
       </c>
-      <c r="J31" s="47" t="s">
+      <c r="J31" s="43" t="s">
         <v>96</v>
       </c>
     </row>
@@ -2744,8 +2758,8 @@
         <v>77</v>
       </c>
       <c r="H32" s="6"/>
-      <c r="I32" s="36"/>
-      <c r="J32" s="47"/>
+      <c r="I32" s="30"/>
+      <c r="J32" s="43"/>
     </row>
     <row r="33" spans="2:10">
       <c r="B33" s="6">
@@ -2754,15 +2768,15 @@
       <c r="C33" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="D33" s="49" t="s">
+      <c r="D33" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="E33" s="50"/>
-      <c r="F33" s="50"/>
-      <c r="G33" s="50"/>
-      <c r="H33" s="50"/>
-      <c r="I33" s="50"/>
-      <c r="J33" s="51"/>
+      <c r="E33" s="26"/>
+      <c r="F33" s="26"/>
+      <c r="G33" s="26"/>
+      <c r="H33" s="26"/>
+      <c r="I33" s="26"/>
+      <c r="J33" s="27"/>
     </row>
     <row r="34" spans="2:10" ht="15" customHeight="1">
       <c r="B34" s="6">
@@ -2784,10 +2798,10 @@
         <v>82</v>
       </c>
       <c r="H34" s="6"/>
-      <c r="I34" s="36" t="s">
+      <c r="I34" s="30" t="s">
         <v>102</v>
       </c>
-      <c r="J34" s="52" t="s">
+      <c r="J34" s="31" t="s">
         <v>105</v>
       </c>
     </row>
@@ -2807,8 +2821,8 @@
         <v>85</v>
       </c>
       <c r="H35" s="6"/>
-      <c r="I35" s="36"/>
-      <c r="J35" s="52"/>
+      <c r="I35" s="30"/>
+      <c r="J35" s="31"/>
     </row>
     <row r="36" spans="2:10">
       <c r="B36" s="6">
@@ -2835,6 +2849,23 @@
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="D25:J25"/>
+    <mergeCell ref="D24:J24"/>
+    <mergeCell ref="I10:I12"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="E10:E12"/>
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="D34:D36"/>
+    <mergeCell ref="E13:E21"/>
+    <mergeCell ref="E26:E32"/>
+    <mergeCell ref="E34:E36"/>
+    <mergeCell ref="D13:D21"/>
+    <mergeCell ref="D26:D32"/>
     <mergeCell ref="J26:J30"/>
     <mergeCell ref="J34:J35"/>
     <mergeCell ref="J3:J4"/>
@@ -2851,23 +2882,6 @@
     <mergeCell ref="I26:I30"/>
     <mergeCell ref="I14:I18"/>
     <mergeCell ref="I31:I32"/>
-    <mergeCell ref="D34:D36"/>
-    <mergeCell ref="E13:E21"/>
-    <mergeCell ref="E26:E32"/>
-    <mergeCell ref="E34:E36"/>
-    <mergeCell ref="D13:D21"/>
-    <mergeCell ref="D26:D32"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="D25:J25"/>
-    <mergeCell ref="D24:J24"/>
-    <mergeCell ref="I10:I12"/>
-    <mergeCell ref="I3:I4"/>
-    <mergeCell ref="E10:E12"/>
-    <mergeCell ref="D5:D7"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E3:H3"/>
-    <mergeCell ref="D3:D4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967294" verticalDpi="0" r:id="rId1"/>
@@ -2888,37 +2902,37 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8">
-      <c r="B2" s="56" t="s">
-        <v>117</v>
-      </c>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
-      <c r="F2" s="57"/>
-      <c r="G2" s="57"/>
-      <c r="H2" s="58"/>
+      <c r="B2" s="54" t="s">
+        <v>115</v>
+      </c>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="56"/>
     </row>
     <row r="3" spans="2:8">
       <c r="B3" s="16" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E3" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="F3" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="G3" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="F3" s="16" t="s">
+      <c r="H3" s="16" t="s">
         <v>114</v>
-      </c>
-      <c r="G3" s="16" t="s">
-        <v>115</v>
-      </c>
-      <c r="H3" s="16" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="4" spans="2:8">
@@ -2926,19 +2940,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H4" s="13">
         <v>12</v>
@@ -2949,19 +2963,19 @@
         <v>2</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H5" s="13">
         <v>1</v>
@@ -2972,19 +2986,19 @@
         <v>3</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H6" s="13">
         <v>2</v>
@@ -2995,19 +3009,19 @@
         <v>4</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H7" s="13">
         <v>3</v>
@@ -3018,19 +3032,19 @@
         <v>5</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H8" s="13">
         <v>4</v>
@@ -3041,19 +3055,19 @@
         <v>6</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D9" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="G9" s="17" t="s">
         <v>129</v>
-      </c>
-      <c r="E9" s="13" t="s">
-        <v>134</v>
-      </c>
-      <c r="F9" s="13" t="s">
-        <v>145</v>
-      </c>
-      <c r="G9" s="17" t="s">
-        <v>131</v>
       </c>
       <c r="H9" s="13">
         <v>5</v>
@@ -3064,19 +3078,19 @@
         <v>7</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H10" s="13">
         <v>11</v>
@@ -3087,19 +3101,19 @@
         <v>8</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H11" s="13">
         <v>10</v>
@@ -3110,19 +3124,19 @@
         <v>9</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G12" s="17" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H12" s="13">
         <v>9</v>
@@ -3133,19 +3147,19 @@
         <v>10</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H13" s="13">
         <v>8</v>
@@ -3156,19 +3170,19 @@
         <v>11</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="G14" s="17" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H14" s="13">
         <v>7</v>
@@ -3179,19 +3193,19 @@
         <v>12</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D15" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="G15" s="17" t="s">
         <v>129</v>
-      </c>
-      <c r="E15" s="13" t="s">
-        <v>135</v>
-      </c>
-      <c r="F15" s="13" t="s">
-        <v>145</v>
-      </c>
-      <c r="G15" s="17" t="s">
-        <v>131</v>
       </c>
       <c r="H15" s="13">
         <v>6</v>
@@ -3202,19 +3216,19 @@
         <v>13</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="G16" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H16" s="13">
         <v>2.5</v>
@@ -3225,19 +3239,19 @@
         <v>14</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="G17" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H17" s="13">
         <v>5</v>
@@ -3248,19 +3262,19 @@
         <v>15</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G18" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H18" s="13">
         <f>H17+2.5</f>
@@ -3272,19 +3286,19 @@
         <v>16</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F19" s="13" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G19" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H19" s="13">
         <f>H18+2.5</f>
@@ -3296,19 +3310,19 @@
         <v>17</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D20" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="F20" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="G20" s="18" t="s">
         <v>128</v>
-      </c>
-      <c r="E20" s="13" t="s">
-        <v>136</v>
-      </c>
-      <c r="F20" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="G20" s="18" t="s">
-        <v>130</v>
       </c>
       <c r="H20" s="13">
         <f>H19+2.5</f>
@@ -3320,19 +3334,19 @@
         <v>18</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G21" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H21" s="13">
         <f>H20+2.5</f>
@@ -3344,19 +3358,19 @@
         <v>19</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F22" s="13" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="G22" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H22" s="13">
         <v>30</v>
@@ -3367,19 +3381,19 @@
         <v>20</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="G23" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H23" s="13">
         <f>H22-2.5</f>
@@ -3391,19 +3405,19 @@
         <v>21</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G24" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H24" s="13">
         <f>H23-2.5</f>
@@ -3415,19 +3429,19 @@
         <v>22</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G25" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H25" s="13">
         <f>H24-2.5</f>
@@ -3439,19 +3453,19 @@
         <v>23</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D26" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="E26" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="F26" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="G26" s="18" t="s">
         <v>128</v>
-      </c>
-      <c r="E26" s="13" t="s">
-        <v>137</v>
-      </c>
-      <c r="F26" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="G26" s="18" t="s">
-        <v>130</v>
       </c>
       <c r="H26" s="13">
         <f>H25-2.5</f>
@@ -3463,19 +3477,19 @@
         <v>24</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F27" s="13" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G27" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H27" s="13">
         <f>H26-2.5</f>
@@ -3487,19 +3501,19 @@
         <v>25</v>
       </c>
       <c r="C28" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D28" s="13" t="s">
         <v>122</v>
       </c>
-      <c r="D28" s="13" t="s">
-        <v>124</v>
-      </c>
       <c r="E28" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="F28" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="F28" s="13" t="s">
-        <v>140</v>
-      </c>
       <c r="G28" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H28" s="13">
         <v>32.5</v>
@@ -3510,19 +3524,19 @@
         <v>26</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="G29" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H29" s="13">
         <f>H28+2.5</f>
@@ -3534,19 +3548,19 @@
         <v>27</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G30" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H30" s="13">
         <f>H29+2.5</f>
@@ -3558,19 +3572,19 @@
         <v>28</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F31" s="13" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G31" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H31" s="13">
         <f>H30+2.5</f>
@@ -3582,19 +3596,19 @@
         <v>29</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D32" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="E32" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="F32" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="G32" s="18" t="s">
         <v>128</v>
-      </c>
-      <c r="E32" s="13" t="s">
-        <v>138</v>
-      </c>
-      <c r="F32" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="G32" s="18" t="s">
-        <v>130</v>
       </c>
       <c r="H32" s="13">
         <f>H31+2.5</f>
@@ -3606,19 +3620,19 @@
         <v>30</v>
       </c>
       <c r="C33" s="13" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D33" s="13" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F33" s="13" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G33" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H33" s="13">
         <f>H32+2.5</f>
@@ -3630,19 +3644,19 @@
         <v>31</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D34" s="13" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F34" s="13" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="G34" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H34" s="13">
         <v>0</v>
@@ -3653,19 +3667,19 @@
         <v>32</v>
       </c>
       <c r="C35" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="D35" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="D35" s="13" t="s">
-        <v>125</v>
-      </c>
       <c r="E35" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="F35" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="F35" s="13" t="s">
-        <v>141</v>
-      </c>
       <c r="G35" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H35" s="13">
         <v>57.5</v>
@@ -3676,19 +3690,19 @@
         <v>33</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F36" s="13" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G36" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H36" s="13">
         <f>H35-2.5</f>
@@ -3700,19 +3714,19 @@
         <v>34</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F37" s="13" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G37" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H37" s="13">
         <f>H36-2.5</f>
@@ -3724,19 +3738,19 @@
         <v>35</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D38" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="E38" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="F38" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="G38" s="18" t="s">
         <v>128</v>
-      </c>
-      <c r="E38" s="13" t="s">
-        <v>139</v>
-      </c>
-      <c r="F38" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="G38" s="18" t="s">
-        <v>130</v>
       </c>
       <c r="H38" s="13">
         <f>H37-2.5</f>
@@ -3748,19 +3762,19 @@
         <v>36</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D39" s="13" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E39" s="13" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F39" s="13" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G39" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H39" s="13">
         <f>H38-2.5</f>

</xml_diff>